<commit_message>
Adding pato imports, preparing imports from sdgio, env, sdc-ontology, revising terms and imports list files
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations /ClimOO Imports.xlsx
+++ b/ClimOO material/materials for implementations /ClimOO Imports.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C570A47F-C514-1345-B8D5-868AC0669903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5731F9-B586-5C4B-996F-9A987338CC11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35460" yWindow="2180" windowWidth="28800" windowHeight="16520" activeTab="2" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
   </bookViews>
   <sheets>
     <sheet name="Ontologies reused" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="324">
   <si>
     <t>Agri-Food Experiment Ontology</t>
   </si>
@@ -992,6 +992,24 @@
   </si>
   <si>
     <t>Giorgio's personal comments</t>
+  </si>
+  <si>
+    <t>Gene Ontology</t>
+  </si>
+  <si>
+    <t>GO</t>
+  </si>
+  <si>
+    <t>https://geneontology.org/</t>
+  </si>
+  <si>
+    <t>PO2</t>
+  </si>
+  <si>
+    <t>https://entrepot.recherche.data.gouv.fr/dataset.xhtml?persistentId=doi:10.15454/XSVVBW</t>
+  </si>
+  <si>
+    <t>Process and Observation Ontology</t>
   </si>
 </sst>
 </file>
@@ -1098,7 +1116,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1169,13 +1187,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1270,6 +1299,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1626,7 +1659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2C20A25-ACC7-684D-AF97-19E64433B7DC}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
@@ -1845,6 +1878,50 @@
         <v>74</v>
       </c>
     </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="36" t="s">
+        <v>318</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>319</v>
+      </c>
+      <c r="C16" s="37" t="s">
+        <v>320</v>
+      </c>
+      <c r="D16" s="36" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="D17" s="36" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="39" t="s">
+        <v>284</v>
+      </c>
+      <c r="B18" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>283</v>
+      </c>
+      <c r="D18" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18"/>
+      <c r="F18"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{8CC07798-E2AF-0146-98EE-D64B8D8E086A}"/>
@@ -1852,6 +1929,9 @@
     <hyperlink ref="C4" r:id="rId3" xr:uid="{42D6353D-9FD9-BB40-801D-3DBBE7A42AD4}"/>
     <hyperlink ref="C5" r:id="rId4" xr:uid="{1723572C-7947-D040-BDA4-751C138A8B77}"/>
     <hyperlink ref="C15" r:id="rId5" xr:uid="{BBA8B89A-7E4D-0C4C-9DCD-9A35275A1053}"/>
+    <hyperlink ref="C16" r:id="rId6" xr:uid="{13BBB7FD-8082-2D42-9493-20D5AF29854A}"/>
+    <hyperlink ref="C17" r:id="rId7" xr:uid="{D3895E0F-1B7A-1C47-B577-5C63E642DBE7}"/>
+    <hyperlink ref="C18" r:id="rId8" xr:uid="{3B5A9A2C-530A-1043-94EC-CC59816CE215}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -1860,7 +1940,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B475128C-F7EE-8540-83D5-7C0DBC4F277D}">
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="37.5" bestFit="1" customWidth="1"/>
@@ -2534,479 +2614,464 @@
         <v>191</v>
       </c>
     </row>
+    <row r="59" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B59" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>175</v>
+      </c>
+    </row>
     <row r="60" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="23" t="s">
-        <v>171</v>
+      <c r="A60" s="8" t="s">
+        <v>166</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C60" s="25" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="61" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B61" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C61" s="9" t="s">
-        <v>175</v>
+      <c r="A61" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="62" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="8" t="s">
-        <v>166</v>
+      <c r="A62" s="23" t="s">
+        <v>104</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C62" s="25" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="B63" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="C63" s="12" t="s">
-        <v>178</v>
+        <v>164</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C63" s="25" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="64" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="B64" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="C64" s="25" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>38</v>
+      <c r="A64" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B65" s="23" t="s">
+        <v>120</v>
       </c>
       <c r="C65" s="25" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
     </row>
     <row r="66" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="21" t="s">
-        <v>284</v>
-      </c>
-      <c r="B66" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="C66" s="30" t="s">
-        <v>283</v>
-      </c>
-      <c r="D66"/>
-      <c r="E66"/>
-      <c r="F66"/>
+      <c r="A66" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="B66" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="C66" s="25" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="67" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B67" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>129</v>
+      <c r="A67" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B67" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C67" s="25" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="68" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B68" s="23" t="s">
-        <v>120</v>
+      <c r="A68" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="B68" s="9" t="s">
+        <v>155</v>
       </c>
       <c r="C68" s="25" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="69" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="B69" s="26" t="s">
-        <v>153</v>
+      <c r="A69" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>157</v>
       </c>
       <c r="C69" s="25" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="70" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B70" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="C70" s="25" t="s">
-        <v>151</v>
-      </c>
+      <c r="A70" s="21" t="s">
+        <v>296</v>
+      </c>
+      <c r="B70" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="C70" s="30" t="s">
+        <v>201</v>
+      </c>
+      <c r="D70"/>
+      <c r="E70"/>
+      <c r="F70"/>
     </row>
     <row r="71" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="23" t="s">
-        <v>107</v>
+        <v>241</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>155</v>
+        <v>242</v>
       </c>
       <c r="C71" s="25" t="s">
-        <v>156</v>
+        <v>240</v>
       </c>
     </row>
     <row r="72" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="B72" s="9" t="s">
-        <v>157</v>
+      <c r="A72" s="21" t="s">
+        <v>239</v>
+      </c>
+      <c r="B72" s="26" t="s">
+        <v>238</v>
       </c>
       <c r="C72" s="25" t="s">
-        <v>156</v>
+        <v>237</v>
       </c>
     </row>
     <row r="73" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="21" t="s">
-        <v>296</v>
-      </c>
-      <c r="B73" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="C73" s="30" t="s">
-        <v>201</v>
-      </c>
-      <c r="D73"/>
-      <c r="E73"/>
-      <c r="F73"/>
+      <c r="A73" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B73" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="C73" s="25" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="74" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="23" t="s">
-        <v>241</v>
+      <c r="A74" s="21" t="s">
+        <v>232</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="C74" s="25" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="75" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="21" t="s">
-        <v>239</v>
-      </c>
-      <c r="B75" s="26" t="s">
-        <v>238</v>
+      <c r="A75" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>5</v>
       </c>
       <c r="C75" s="25" t="s">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="76" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="B76" s="26" t="s">
-        <v>236</v>
+      <c r="A76" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="B76" s="9" t="s">
+        <v>173</v>
       </c>
       <c r="C76" s="25" t="s">
-        <v>235</v>
+        <v>174</v>
       </c>
     </row>
     <row r="77" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="21" t="s">
-        <v>232</v>
-      </c>
-      <c r="B77" s="9" t="s">
-        <v>233</v>
+      <c r="A77" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>45</v>
       </c>
       <c r="C77" s="25" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C78" s="25" t="s">
-        <v>269</v>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B78" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="C78" s="9" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="79" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="B79" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="C79" s="25" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C80" s="25" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="B81" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C81" s="9" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B79" s="9"/>
+      <c r="C79" s="9" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" s="7" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="B81" s="12"/>
+      <c r="C81" s="13" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="B82" s="9"/>
-      <c r="C82" s="9" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" s="7" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="16" t="s">
-        <v>15</v>
+        <v>96</v>
+      </c>
+      <c r="B82" s="12"/>
+      <c r="C82" s="25" t="s">
+        <v>243</v>
+      </c>
+      <c r="D82" s="7"/>
+      <c r="E82" s="7"/>
+      <c r="F82" s="7"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A83" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="B84" s="12"/>
-      <c r="C84" s="13" t="s">
-        <v>244</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="D83" s="7"/>
+      <c r="E83" s="7"/>
+      <c r="F83" s="7"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A84" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D84" s="7"/>
+      <c r="E84" s="7"/>
+      <c r="F84" s="7"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A85" s="23" t="s">
-        <v>96</v>
+      <c r="A85" s="21" t="s">
+        <v>98</v>
       </c>
       <c r="B85" s="12"/>
       <c r="C85" s="25" t="s">
-        <v>243</v>
+        <v>194</v>
       </c>
       <c r="D85" s="7"/>
-      <c r="E85" s="7"/>
+      <c r="E85" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F85" s="7"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A86" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B86" s="4"/>
-      <c r="C86" s="4" t="s">
-        <v>201</v>
+      <c r="A86" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B86" s="12"/>
+      <c r="C86" s="25" t="s">
+        <v>189</v>
       </c>
       <c r="D86" s="7"/>
       <c r="E86" s="7"/>
       <c r="F86" s="7"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A87" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="B87" s="4"/>
-      <c r="C87" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D87" s="7"/>
+      <c r="A87" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="B87" s="12"/>
+      <c r="C87" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="E87" s="7"/>
       <c r="F87" s="7"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A88" s="21" t="s">
-        <v>98</v>
+      <c r="A88" s="23" t="s">
+        <v>100</v>
       </c>
       <c r="B88" s="12"/>
       <c r="C88" s="25" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="D88" s="7"/>
-      <c r="E88" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="E88" s="7"/>
       <c r="F88" s="7"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A89" s="8" t="s">
-        <v>99</v>
+      <c r="A89" s="23" t="s">
+        <v>103</v>
       </c>
       <c r="B89" s="12"/>
       <c r="C89" s="25" t="s">
-        <v>189</v>
+        <v>165</v>
       </c>
       <c r="D89" s="7"/>
       <c r="E89" s="7"/>
       <c r="F89" s="7"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A90" s="23" t="s">
-        <v>102</v>
+      <c r="A90" s="15" t="s">
+        <v>105</v>
       </c>
       <c r="B90" s="12"/>
       <c r="C90" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="D90" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="D90" s="7"/>
       <c r="E90" s="7"/>
       <c r="F90" s="7"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A91" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="B91" s="12"/>
-      <c r="C91" s="25" t="s">
-        <v>176</v>
-      </c>
-      <c r="D91" s="7"/>
-      <c r="E91" s="7"/>
-      <c r="F91" s="7"/>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A92" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="B92" s="12"/>
-      <c r="C92" s="25" t="s">
-        <v>165</v>
-      </c>
-      <c r="D92" s="7"/>
-      <c r="E92" s="7"/>
-      <c r="F92" s="7"/>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A93" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="B93" s="12"/>
-      <c r="C93" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="D93" s="7"/>
-      <c r="E93" s="7"/>
-      <c r="F93" s="7"/>
+      <c r="A91" t="s">
+        <v>323</v>
+      </c>
+      <c r="B91" t="s">
+        <v>321</v>
+      </c>
+      <c r="C91" s="38" t="s">
+        <v>322</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F93">
-    <sortCondition ref="B3:B93"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F90">
+    <sortCondition ref="B3:B90"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="C11" r:id="rId1" xr:uid="{0516338A-57C0-AF4C-9903-653CC3B4F1C5}"/>
     <hyperlink ref="C16" r:id="rId2" xr:uid="{842A1859-6DEA-3341-A7EE-DAA84D26CB75}"/>
     <hyperlink ref="C15" r:id="rId3" xr:uid="{2C9FEB54-CD6A-5A43-8855-AD56B398AEBC}"/>
     <hyperlink ref="C28" r:id="rId4" xr:uid="{E16A0D71-DA2F-B04F-8D58-A68F854A57F9}"/>
-    <hyperlink ref="C67" r:id="rId5" xr:uid="{C6F40C8D-7190-B740-B426-605371E8ECF8}"/>
+    <hyperlink ref="C64" r:id="rId5" xr:uid="{C6F40C8D-7190-B740-B426-605371E8ECF8}"/>
     <hyperlink ref="C47" r:id="rId6" xr:uid="{A4D49E13-D104-8649-9EC7-2550F793CAD4}"/>
     <hyperlink ref="C54" r:id="rId7" xr:uid="{B787D633-212B-B248-9307-3E1160DF1616}"/>
     <hyperlink ref="A30" r:id="rId8" display="https://ecoportal.lifewatch.eu/ontologies/ECSO" xr:uid="{489A4471-C877-F24D-930D-E81D9F374810}"/>
     <hyperlink ref="A23" r:id="rId9" display="https://ecoportal.lifewatch.eu/ontologies/CPMETA" xr:uid="{F56D74CE-A25A-D945-B0FC-F5827574981B}"/>
     <hyperlink ref="A32" r:id="rId10" display="https://biodivportal.gfbio.org/ontologies/EDAM" xr:uid="{05E273E9-A029-9643-A707-D384B4637DC0}"/>
-    <hyperlink ref="A62" r:id="rId11" display="https://biodivportal.gfbio.org/ontologies/QUDT" xr:uid="{9C2C2B49-4FA5-224C-8CDA-C2FF9E132E7B}"/>
+    <hyperlink ref="A60" r:id="rId11" display="https://biodivportal.gfbio.org/ontologies/QUDT" xr:uid="{9C2C2B49-4FA5-224C-8CDA-C2FF9E132E7B}"/>
     <hyperlink ref="A27" r:id="rId12" display="https://biodivportal.gfbio.org/ontologies/ECO" xr:uid="{B297B450-7DF2-BE4D-92C9-78500CB10ED6}"/>
     <hyperlink ref="A45" r:id="rId13" display="https://agroportal.lirmm.fr/ontologies/INRAETHES" xr:uid="{C71C31BE-87FF-0540-B26B-F6CEFAB9E223}"/>
-    <hyperlink ref="A79" r:id="rId14" display="https://agroportal.lirmm.fr/ontologies/TRANSFORMON" xr:uid="{7900C719-E36D-9F49-A23A-081FF403C10B}"/>
+    <hyperlink ref="A76" r:id="rId14" display="https://agroportal.lirmm.fr/ontologies/TRANSFORMON" xr:uid="{7900C719-E36D-9F49-A23A-081FF403C10B}"/>
     <hyperlink ref="A8" r:id="rId15" display="https://agroportal.lirmm.fr/ontologies/AGRONTOLOGY" xr:uid="{22EC63C0-9A81-6045-B4AD-452C2F098677}"/>
     <hyperlink ref="A22" r:id="rId16" display="https://scs-ontouml.eemcs.utwente.nl/model/ef85708e-02ce-40b4-8fdb-57799201ee28" xr:uid="{A0736C9C-D991-7E40-966A-7E4DBD6E9F8B}"/>
-    <hyperlink ref="A89" r:id="rId17" display="https://scs-ontouml.eemcs.utwente.nl/model/87dea242-75d9-4b89-99f3-6f52c0855f3a" xr:uid="{15A93492-DAFA-2845-8CC5-6AA56A81A3CD}"/>
-    <hyperlink ref="A93" r:id="rId18" display="https://scs-ontouml.eemcs.utwente.nl/model/06130cd9-ba26-4324-9f1e-88bd03b88ca9" xr:uid="{C8F0AAC8-E15C-1C40-84AD-77046731CC14}"/>
+    <hyperlink ref="A86" r:id="rId17" display="https://scs-ontouml.eemcs.utwente.nl/model/87dea242-75d9-4b89-99f3-6f52c0855f3a" xr:uid="{15A93492-DAFA-2845-8CC5-6AA56A81A3CD}"/>
+    <hyperlink ref="A90" r:id="rId18" display="https://scs-ontouml.eemcs.utwente.nl/model/06130cd9-ba26-4324-9f1e-88bd03b88ca9" xr:uid="{C8F0AAC8-E15C-1C40-84AD-77046731CC14}"/>
     <hyperlink ref="A52" r:id="rId19" display="https://earthportal.eu/ontologies/NVS_P07" xr:uid="{736D9821-6418-B042-A265-9F93FEBFC2AB}"/>
     <hyperlink ref="B20" r:id="rId20" display="https://ontobee.org/ontology/CHMO" xr:uid="{D80FD32C-0186-074E-A789-BA63C3C0FBA2}"/>
-    <hyperlink ref="C93" r:id="rId21" xr:uid="{FA229F1B-6A23-4D4F-9F4B-A36373D74F93}"/>
+    <hyperlink ref="C90" r:id="rId21" xr:uid="{FA229F1B-6A23-4D4F-9F4B-A36373D74F93}"/>
     <hyperlink ref="C17" r:id="rId22" xr:uid="{C2E8234F-2FE4-6F42-B474-076224A40CF9}"/>
-    <hyperlink ref="C80" r:id="rId23" xr:uid="{9D2AB138-A508-0C43-BF5D-6A7912111510}"/>
+    <hyperlink ref="C77" r:id="rId23" xr:uid="{9D2AB138-A508-0C43-BF5D-6A7912111510}"/>
     <hyperlink ref="C25" r:id="rId24" xr:uid="{B570D235-B996-7644-80AC-4CD5B56BE905}"/>
     <hyperlink ref="C46" r:id="rId25" location="IntegrationTime" xr:uid="{5959054A-F7E7-8542-8583-0A4558203518}"/>
     <hyperlink ref="C48" r:id="rId26" location="IntegrationTime" xr:uid="{1A64D5B5-27D6-CF42-BC35-2479D2C36AED}"/>
     <hyperlink ref="C2" r:id="rId27" xr:uid="{555FFEC9-5DBF-7E47-A4C5-DF9FC5B70EEF}"/>
     <hyperlink ref="C30" r:id="rId28" xr:uid="{8104D6FC-1ECF-DC4C-8655-94D174EC37CC}"/>
-    <hyperlink ref="C65" r:id="rId29" xr:uid="{1C9B4C0D-6549-CD44-B478-E27B648E157F}"/>
+    <hyperlink ref="C63" r:id="rId29" xr:uid="{1C9B4C0D-6549-CD44-B478-E27B648E157F}"/>
     <hyperlink ref="C24" r:id="rId30" xr:uid="{A852BE4A-D08B-6946-B29D-45CBCF0394DD}"/>
-    <hyperlink ref="C70" r:id="rId31" xr:uid="{3B72C5B5-48F0-1E46-A319-25228DF071D2}"/>
-    <hyperlink ref="C71" r:id="rId32" xr:uid="{AB328289-A6B1-A24B-8D21-A5BEBDD8F017}"/>
-    <hyperlink ref="C72" r:id="rId33" xr:uid="{F2496C0E-1F74-1443-B9AA-12A2AA4BD022}"/>
+    <hyperlink ref="C67" r:id="rId31" xr:uid="{3B72C5B5-48F0-1E46-A319-25228DF071D2}"/>
+    <hyperlink ref="C68" r:id="rId32" xr:uid="{AB328289-A6B1-A24B-8D21-A5BEBDD8F017}"/>
+    <hyperlink ref="C69" r:id="rId33" xr:uid="{F2496C0E-1F74-1443-B9AA-12A2AA4BD022}"/>
     <hyperlink ref="C51" r:id="rId34" xr:uid="{1A706F58-35D7-0542-8C3B-2D83812A6BC4}"/>
-    <hyperlink ref="C68" r:id="rId35" xr:uid="{634BD972-B958-864D-A34A-ED64E1A54F14}"/>
-    <hyperlink ref="C64" r:id="rId36" xr:uid="{40641FB9-AD2F-1A47-8768-874BF77204F6}"/>
-    <hyperlink ref="C92" r:id="rId37" xr:uid="{E0E26C66-761F-854D-979B-011E460B7BB4}"/>
-    <hyperlink ref="C62" r:id="rId38" xr:uid="{BEF1E317-B39A-4C41-A822-29A9E0AECDC6}"/>
-    <hyperlink ref="C60" r:id="rId39" xr:uid="{D3895E0F-1B7A-1C47-B577-5C63E642DBE7}"/>
-    <hyperlink ref="C79" r:id="rId40" xr:uid="{FFDDE5B3-5EE4-1749-9283-B2404C450D47}"/>
-    <hyperlink ref="C91" r:id="rId41" xr:uid="{DBB12542-F692-2D44-8CC1-2B25F55AAD71}"/>
-    <hyperlink ref="C56" r:id="rId42" xr:uid="{5987C402-1AD0-6D41-A7D9-03F070A22118}"/>
-    <hyperlink ref="C55" r:id="rId43" xr:uid="{150DE845-C329-BE4C-8356-8A23832BDA6C}"/>
-    <hyperlink ref="C32" r:id="rId44" xr:uid="{42A2ED53-4748-F144-8042-83EA3FAEFFA5}"/>
-    <hyperlink ref="C90" r:id="rId45" xr:uid="{34A568F4-314D-DC45-9FCD-09BA8D852696}"/>
-    <hyperlink ref="C89" r:id="rId46" xr:uid="{6B71E233-8757-2F44-9B59-3AC56BC52D0C}"/>
-    <hyperlink ref="C57" r:id="rId47" xr:uid="{16A8DEC0-BB7C-9E4A-98B5-FCE7FCC17235}"/>
-    <hyperlink ref="C58" r:id="rId48" xr:uid="{05EB2E2A-9E63-E44D-A471-922CC35999FF}"/>
-    <hyperlink ref="C88" r:id="rId49" xr:uid="{37DA00E0-DBDE-954F-8690-A8F468128B22}"/>
-    <hyperlink ref="C50" r:id="rId50" xr:uid="{39E38128-6CD3-4F43-9AC7-CF7D9BE6C2A7}"/>
-    <hyperlink ref="C49" r:id="rId51" xr:uid="{CC63136F-DDDE-0E4A-9C74-5CF0B3DA4AE0}"/>
-    <hyperlink ref="C42" r:id="rId52" xr:uid="{D64E825D-1515-7747-B40D-8BB67687D95E}"/>
-    <hyperlink ref="C41" r:id="rId53" xr:uid="{FC234C3F-958C-5D40-B086-278A90BA0EF1}"/>
-    <hyperlink ref="C31" r:id="rId54" xr:uid="{695DC735-428C-B641-B857-BE4BABD039B4}"/>
-    <hyperlink ref="C33" r:id="rId55" xr:uid="{A6123D3B-9344-4648-A798-C9656105EC8E}"/>
-    <hyperlink ref="C27" r:id="rId56" xr:uid="{FAC8521C-4FCA-F948-A085-6440C8E00231}"/>
-    <hyperlink ref="C37" r:id="rId57" xr:uid="{D38C8FF9-E399-C041-A2E3-AFB79B4566B1}"/>
-    <hyperlink ref="C36" r:id="rId58" xr:uid="{F63B92C4-2FC2-4D43-8C6F-9C661D780DD5}"/>
-    <hyperlink ref="C35" r:id="rId59" xr:uid="{A571D68F-535D-D14F-8880-19F19B69EEE5}"/>
-    <hyperlink ref="C26" r:id="rId60" xr:uid="{C22900F2-9599-4B45-A290-FB71BBD4FF5B}"/>
-    <hyperlink ref="C29" r:id="rId61" xr:uid="{8223A1A7-D0DE-AA4B-B603-47062E37F784}"/>
-    <hyperlink ref="C77" r:id="rId62" xr:uid="{491775E5-F6D6-3C4D-BA3E-FDF22E9AB107}"/>
-    <hyperlink ref="C76" r:id="rId63" xr:uid="{F6DAB0F7-E03C-6244-A128-6CA285F0E2A4}"/>
-    <hyperlink ref="C75" r:id="rId64" xr:uid="{17948612-13E1-F149-93B9-52D5F110C470}"/>
-    <hyperlink ref="C74" r:id="rId65" xr:uid="{E4A8AFB7-C66A-3240-BF7D-F2916C093943}"/>
-    <hyperlink ref="C85" r:id="rId66" xr:uid="{C497F7E2-44E7-6E4C-9415-4899C4175F6C}"/>
-    <hyperlink ref="C21" r:id="rId67" xr:uid="{7BC2260B-5940-E74A-A602-B4B86FC797AF}"/>
-    <hyperlink ref="C22" r:id="rId68" xr:uid="{9C45F978-C4FF-5048-930F-BE11F56D1C53}"/>
-    <hyperlink ref="C20" r:id="rId69" xr:uid="{80DD7C05-67E3-0740-BF49-6E58E3E96F3C}"/>
-    <hyperlink ref="C18" r:id="rId70" xr:uid="{1AC78E80-6D26-9741-B8D8-341DC6142958}"/>
-    <hyperlink ref="C12" r:id="rId71" xr:uid="{87AABB3A-A36D-5A42-9490-9C02BDBF3ACA}"/>
-    <hyperlink ref="C10" r:id="rId72" xr:uid="{EE9AD4F8-3C82-DB49-B3CF-9DEC32F45D34}"/>
-    <hyperlink ref="C8" r:id="rId73" xr:uid="{10AD49BC-9BE8-D049-95CD-2C518E2353F0}"/>
-    <hyperlink ref="C13" r:id="rId74" xr:uid="{4370A7CB-AB57-B84F-9241-5D6324A48F1A}"/>
-    <hyperlink ref="C78" r:id="rId75" xr:uid="{A5AA1886-54E0-5149-AE81-CBA997AA90AF}"/>
-    <hyperlink ref="C3" r:id="rId76" xr:uid="{A0E7AA6A-89DB-EC4B-8836-4EC86341F9DD}"/>
-    <hyperlink ref="C7" r:id="rId77" xr:uid="{32CD64DA-7FE0-7B40-A2C5-15EC589F8D17}"/>
-    <hyperlink ref="C4" r:id="rId78" xr:uid="{6CF857B4-8FB8-114F-8A69-4AD1B1F35974}"/>
-    <hyperlink ref="C66" r:id="rId79" xr:uid="{3B5A9A2C-530A-1043-94EC-CC59816CE215}"/>
-    <hyperlink ref="C9" r:id="rId80" xr:uid="{7136ECA6-283D-874C-B90C-8E7F28251500}"/>
-    <hyperlink ref="C39" r:id="rId81" xr:uid="{5D63D260-C4DB-6F4A-ADEC-AF6FBC11A7DD}"/>
+    <hyperlink ref="C65" r:id="rId35" xr:uid="{634BD972-B958-864D-A34A-ED64E1A54F14}"/>
+    <hyperlink ref="C62" r:id="rId36" xr:uid="{40641FB9-AD2F-1A47-8768-874BF77204F6}"/>
+    <hyperlink ref="C89" r:id="rId37" xr:uid="{E0E26C66-761F-854D-979B-011E460B7BB4}"/>
+    <hyperlink ref="C60" r:id="rId38" xr:uid="{BEF1E317-B39A-4C41-A822-29A9E0AECDC6}"/>
+    <hyperlink ref="C76" r:id="rId39" xr:uid="{FFDDE5B3-5EE4-1749-9283-B2404C450D47}"/>
+    <hyperlink ref="C88" r:id="rId40" xr:uid="{DBB12542-F692-2D44-8CC1-2B25F55AAD71}"/>
+    <hyperlink ref="C56" r:id="rId41" xr:uid="{5987C402-1AD0-6D41-A7D9-03F070A22118}"/>
+    <hyperlink ref="C55" r:id="rId42" xr:uid="{150DE845-C329-BE4C-8356-8A23832BDA6C}"/>
+    <hyperlink ref="C32" r:id="rId43" xr:uid="{42A2ED53-4748-F144-8042-83EA3FAEFFA5}"/>
+    <hyperlink ref="C87" r:id="rId44" xr:uid="{34A568F4-314D-DC45-9FCD-09BA8D852696}"/>
+    <hyperlink ref="C86" r:id="rId45" xr:uid="{6B71E233-8757-2F44-9B59-3AC56BC52D0C}"/>
+    <hyperlink ref="C57" r:id="rId46" xr:uid="{16A8DEC0-BB7C-9E4A-98B5-FCE7FCC17235}"/>
+    <hyperlink ref="C58" r:id="rId47" xr:uid="{05EB2E2A-9E63-E44D-A471-922CC35999FF}"/>
+    <hyperlink ref="C85" r:id="rId48" xr:uid="{37DA00E0-DBDE-954F-8690-A8F468128B22}"/>
+    <hyperlink ref="C50" r:id="rId49" xr:uid="{39E38128-6CD3-4F43-9AC7-CF7D9BE6C2A7}"/>
+    <hyperlink ref="C49" r:id="rId50" xr:uid="{CC63136F-DDDE-0E4A-9C74-5CF0B3DA4AE0}"/>
+    <hyperlink ref="C42" r:id="rId51" xr:uid="{D64E825D-1515-7747-B40D-8BB67687D95E}"/>
+    <hyperlink ref="C41" r:id="rId52" xr:uid="{FC234C3F-958C-5D40-B086-278A90BA0EF1}"/>
+    <hyperlink ref="C31" r:id="rId53" xr:uid="{695DC735-428C-B641-B857-BE4BABD039B4}"/>
+    <hyperlink ref="C33" r:id="rId54" xr:uid="{A6123D3B-9344-4648-A798-C9656105EC8E}"/>
+    <hyperlink ref="C27" r:id="rId55" xr:uid="{FAC8521C-4FCA-F948-A085-6440C8E00231}"/>
+    <hyperlink ref="C37" r:id="rId56" xr:uid="{D38C8FF9-E399-C041-A2E3-AFB79B4566B1}"/>
+    <hyperlink ref="C36" r:id="rId57" xr:uid="{F63B92C4-2FC2-4D43-8C6F-9C661D780DD5}"/>
+    <hyperlink ref="C35" r:id="rId58" xr:uid="{A571D68F-535D-D14F-8880-19F19B69EEE5}"/>
+    <hyperlink ref="C26" r:id="rId59" xr:uid="{C22900F2-9599-4B45-A290-FB71BBD4FF5B}"/>
+    <hyperlink ref="C29" r:id="rId60" xr:uid="{8223A1A7-D0DE-AA4B-B603-47062E37F784}"/>
+    <hyperlink ref="C74" r:id="rId61" xr:uid="{491775E5-F6D6-3C4D-BA3E-FDF22E9AB107}"/>
+    <hyperlink ref="C73" r:id="rId62" xr:uid="{F6DAB0F7-E03C-6244-A128-6CA285F0E2A4}"/>
+    <hyperlink ref="C72" r:id="rId63" xr:uid="{17948612-13E1-F149-93B9-52D5F110C470}"/>
+    <hyperlink ref="C71" r:id="rId64" xr:uid="{E4A8AFB7-C66A-3240-BF7D-F2916C093943}"/>
+    <hyperlink ref="C82" r:id="rId65" xr:uid="{C497F7E2-44E7-6E4C-9415-4899C4175F6C}"/>
+    <hyperlink ref="C21" r:id="rId66" xr:uid="{7BC2260B-5940-E74A-A602-B4B86FC797AF}"/>
+    <hyperlink ref="C22" r:id="rId67" xr:uid="{9C45F978-C4FF-5048-930F-BE11F56D1C53}"/>
+    <hyperlink ref="C20" r:id="rId68" xr:uid="{80DD7C05-67E3-0740-BF49-6E58E3E96F3C}"/>
+    <hyperlink ref="C18" r:id="rId69" xr:uid="{1AC78E80-6D26-9741-B8D8-341DC6142958}"/>
+    <hyperlink ref="C12" r:id="rId70" xr:uid="{87AABB3A-A36D-5A42-9490-9C02BDBF3ACA}"/>
+    <hyperlink ref="C10" r:id="rId71" xr:uid="{EE9AD4F8-3C82-DB49-B3CF-9DEC32F45D34}"/>
+    <hyperlink ref="C8" r:id="rId72" xr:uid="{10AD49BC-9BE8-D049-95CD-2C518E2353F0}"/>
+    <hyperlink ref="C13" r:id="rId73" xr:uid="{4370A7CB-AB57-B84F-9241-5D6324A48F1A}"/>
+    <hyperlink ref="C75" r:id="rId74" xr:uid="{A5AA1886-54E0-5149-AE81-CBA997AA90AF}"/>
+    <hyperlink ref="C3" r:id="rId75" xr:uid="{A0E7AA6A-89DB-EC4B-8836-4EC86341F9DD}"/>
+    <hyperlink ref="C7" r:id="rId76" xr:uid="{32CD64DA-7FE0-7B40-A2C5-15EC589F8D17}"/>
+    <hyperlink ref="C4" r:id="rId77" xr:uid="{6CF857B4-8FB8-114F-8A69-4AD1B1F35974}"/>
+    <hyperlink ref="C9" r:id="rId78" xr:uid="{7136ECA6-283D-874C-B90C-8E7F28251500}"/>
+    <hyperlink ref="C39" r:id="rId79" xr:uid="{5D63D260-C4DB-6F4A-ADEC-AF6FBC11A7DD}"/>
+    <hyperlink ref="C91" r:id="rId80" xr:uid="{EAA5189B-F422-1246-8B84-C62DB7CF2462}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Revisions import and vocabulary lists
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations /ClimOO Imports.xlsx
+++ b/ClimOO material/materials for implementations /ClimOO Imports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A265FE2-2DDF-824F-888B-B84FE1B7FB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B505C8-95BF-3F40-A072-6F125F8AC27C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16420" activeTab="1" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" activeTab="1" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
   </bookViews>
   <sheets>
     <sheet name="Ontologies reused" sheetId="3" r:id="rId1"/>
@@ -1297,7 +1297,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1388,16 +1388,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -2139,7 +2137,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="39" t="s">
+      <c r="A8" t="s">
         <v>347</v>
       </c>
       <c r="B8" s="8" t="s">
@@ -2283,7 +2281,7 @@
       <c r="A20" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="39" t="s">
+      <c r="B20" t="s">
         <v>106</v>
       </c>
       <c r="C20" s="23" t="s">
@@ -2305,7 +2303,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="39" t="s">
+      <c r="A22" t="s">
         <v>88</v>
       </c>
       <c r="B22" s="8" t="s">
@@ -2316,13 +2314,13 @@
       </c>
     </row>
     <row r="23" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="39" t="s">
+      <c r="A23" t="s">
         <v>174</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="C23" s="40" t="s">
+      <c r="C23" s="36" t="s">
         <v>342</v>
       </c>
       <c r="D23" s="6" t="s">
@@ -2369,7 +2367,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="39" t="s">
+      <c r="A27" t="s">
         <v>346</v>
       </c>
       <c r="B27" s="8" t="s">
@@ -2402,7 +2400,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="41" t="s">
+      <c r="A30" s="37" t="s">
         <v>345</v>
       </c>
       <c r="B30" s="8" t="s">
@@ -2424,7 +2422,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="39" t="s">
+      <c r="A32" t="s">
         <v>344</v>
       </c>
       <c r="B32" s="8" t="s">
@@ -2573,7 +2571,7 @@
       </c>
     </row>
     <row r="45" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="39" t="s">
+      <c r="A45" t="s">
         <v>191</v>
       </c>
       <c r="B45" s="8" t="s">
@@ -2650,7 +2648,7 @@
       </c>
     </row>
     <row r="52" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="39" t="s">
+      <c r="A52" t="s">
         <v>243</v>
       </c>
       <c r="B52" s="20" t="s">
@@ -2738,7 +2736,7 @@
       </c>
     </row>
     <row r="60" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="39" t="s">
+      <c r="A60" t="s">
         <v>160</v>
       </c>
       <c r="B60" s="8" t="s">
@@ -2917,7 +2915,7 @@
       </c>
     </row>
     <row r="76" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="39" t="s">
+      <c r="A76" t="s">
         <v>166</v>
       </c>
       <c r="B76" s="8" t="s">
@@ -3029,7 +3027,7 @@
       <c r="F85" s="6"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A86" s="39" t="s">
+      <c r="A86" t="s">
         <v>94</v>
       </c>
       <c r="B86" s="11"/>
@@ -3079,7 +3077,7 @@
       <c r="F89" s="6"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A90" s="39" t="s">
+      <c r="A90" s="21" t="s">
         <v>100</v>
       </c>
       <c r="B90" s="11"/>
@@ -3091,24 +3089,24 @@
       <c r="F90" s="6"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+      <c r="A91" s="21" t="s">
         <v>316</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="21" t="s">
         <v>314</v>
       </c>
-      <c r="C91" s="36" t="s">
+      <c r="C91" s="28" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+      <c r="A92" s="21" t="s">
         <v>318</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="21" t="s">
         <v>317</v>
       </c>
-      <c r="C92" s="36" t="s">
+      <c r="C92" s="28" t="s">
         <v>319</v>
       </c>
       <c r="D92" t="s">
@@ -3116,13 +3114,13 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
+      <c r="A93" s="21" t="s">
         <v>320</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="21" t="s">
         <v>321</v>
       </c>
-      <c r="C93" s="36" t="s">
+      <c r="C93" s="28" t="s">
         <v>353</v>
       </c>
       <c r="D93" t="s">
@@ -3130,24 +3128,24 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+      <c r="A94" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="21" t="s">
         <v>322</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C94" s="21" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A95" s="37" t="s">
+      <c r="A95" s="38" t="s">
         <v>326</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="21" t="s">
         <v>325</v>
       </c>
-      <c r="C95" s="36" t="s">
+      <c r="C95" s="28" t="s">
         <v>327</v>
       </c>
       <c r="D95" t="s">
@@ -3155,13 +3153,13 @@
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A96" s="34" t="s">
+      <c r="A96" s="21" t="s">
         <v>328</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="21" t="s">
         <v>329</v>
       </c>
-      <c r="C96" s="36" t="s">
+      <c r="C96" s="28" t="s">
         <v>352</v>
       </c>
       <c r="D96" t="s">
@@ -3169,65 +3167,66 @@
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
+      <c r="A97" s="21" t="s">
         <v>332</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="21" t="s">
         <v>331</v>
       </c>
-      <c r="C97" t="s">
+      <c r="C97" s="21" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="A98" s="38" t="s">
+    <row r="98" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A98" s="39" t="s">
         <v>335</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="21" t="s">
         <v>333</v>
       </c>
-      <c r="C98" s="36" t="s">
+      <c r="C98" s="28" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
+      <c r="A99" s="21" t="s">
         <v>337</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="21" t="s">
         <v>336</v>
       </c>
-      <c r="C99" s="36" t="s">
+      <c r="C99" s="28" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+      <c r="A100" s="21" t="s">
         <v>340</v>
       </c>
-      <c r="C100" s="36" t="s">
+      <c r="B100" s="21"/>
+      <c r="C100" s="28" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A101" s="38" t="s">
+      <c r="A101" s="39" t="s">
         <v>349</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="21" t="s">
         <v>348</v>
       </c>
-      <c r="C101" s="36" t="s">
+      <c r="C101" s="28" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
+      <c r="A102" s="21" t="s">
         <v>282</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="21" t="s">
         <v>283</v>
       </c>
-      <c r="C102" s="36" t="s">
+      <c r="C102" s="28" t="s">
         <v>351</v>
       </c>
     </row>

</xml_diff>